<commit_message>
Update CLS benchmark artifacts
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.4.2/multi_label_cls/MULTI_LABEL_CLS-high-level-summary.xlsx
+++ b/tests/perf_v2/perf_history/v2.4.2/multi_label_cls/MULTI_LABEL_CLS-high-level-summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH6"/>
+  <dimension ref="A1:AH5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,152 +446,152 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>training:epoch_mean</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>training:epoch_std</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>training:e2e_time_mean</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>training:e2e_time_std</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>training:gpu_mem_mean</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>training:gpu_mem_std</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>training:val/accuracy_mean</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>training:val/accuracy_std</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>training:train/iter_time_mean</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>training:train/iter_time_std</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>optimize:e2e_time_mean</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>optimize:e2e_time_std</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>export:test/accuracy_mean</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>export:test/accuracy_std</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>export:test/latency_mean</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>export:test/latency_std</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>export:test/e2e_time_mean</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>export:test/e2e_time_std</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/accuracy_mean</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/accuracy_std</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/iter_time_mean</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/iter_time_std</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/latency_mean</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>torch:test/latency_std</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/accuracy_mean</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/accuracy_std</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/latency_mean</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/latency_std</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/e2e_time_mean</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>optimize:test/e2e_time_std</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/accuracy_mean</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/accuracy_std</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/iter_time_mean</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/iter_time_std</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/latency_mean</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>torch:test/latency_std</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>training:epoch_mean</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>training:epoch_std</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>training:e2e_time_mean</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>training:e2e_time_std</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>training:gpu_mem_mean</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>training:gpu_mem_std</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>training:val/accuracy_mean</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>training:val/accuracy_std</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>training:train/iter_time_mean</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>training:train/iter_time_std</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>optimize:e2e_time_mean</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>optimize:e2e_time_std</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
@@ -617,94 +617,94 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.8588</v>
+        <v>76.25</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0428</v>
+        <v>29.9682</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0215</v>
+        <v>78.99679999999999</v>
       </c>
       <c r="G2" t="n">
+        <v>64.4455</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.5025</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.4328</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.8963</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0452</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.017</v>
+      </c>
+      <c r="N2" t="n">
+        <v>15.736</v>
+      </c>
+      <c r="O2" t="n">
+        <v>7.1507</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0495</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.0209</v>
+      </c>
+      <c r="S2" t="n">
         <v>0.0046</v>
       </c>
-      <c r="H2" t="n">
-        <v>3.4032</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.9115</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.8575</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.0428</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.0286</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.0076</v>
-      </c>
-      <c r="N2" t="n">
-        <v>4.4165</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.9591</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.8586</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0428</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.06419999999999999</v>
-      </c>
       <c r="T2" t="n">
-        <v>0.0135</v>
+        <v>3.2912</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0037</v>
+        <v>0.8421999999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>76.40000000000001</v>
+        <v>0.8541</v>
       </c>
       <c r="W2" t="n">
-        <v>26.7668</v>
+        <v>0.0487</v>
       </c>
       <c r="X2" t="n">
-        <v>91.6596</v>
+        <v>0.0721</v>
       </c>
       <c r="Y2" t="n">
-        <v>69.2831</v>
+        <v>0.0603</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.447</v>
+        <v>0.0121</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.3908</v>
+        <v>0.0032</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.8954</v>
+        <v>0.8512</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.0479</v>
+        <v>0.0497</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.0742</v>
+        <v>0.0284</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.0248</v>
+        <v>0.0074</v>
       </c>
       <c r="AF2" t="n">
-        <v>17.3302</v>
+        <v>4.3882</v>
       </c>
       <c r="AG2" t="n">
-        <v>8.17</v>
+        <v>0.9506</v>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
@@ -729,94 +729,94 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.8557</v>
+        <v>69.45</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0409</v>
+        <v>18.0656</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0189</v>
+        <v>79.5087</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0043</v>
+        <v>65.042</v>
       </c>
       <c r="H3" t="n">
-        <v>3.0552</v>
+        <v>3.6615</v>
       </c>
       <c r="I3" t="n">
-        <v>0.8013</v>
+        <v>1.174</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8535</v>
+        <v>0.8994</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0417</v>
+        <v>0.0511</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0235</v>
+        <v>0.07969999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0048</v>
+        <v>0.0091</v>
       </c>
       <c r="N3" t="n">
-        <v>3.8195</v>
+        <v>12.1395</v>
       </c>
       <c r="O3" t="n">
-        <v>1.0486</v>
+        <v>5.7387</v>
       </c>
       <c r="P3" t="n">
-        <v>0.8552</v>
+        <v>0.8516</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0402</v>
+        <v>0.0394</v>
       </c>
       <c r="R3" t="n">
-        <v>0.1028</v>
+        <v>0.0193</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0489</v>
+        <v>0.0041</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0124</v>
+        <v>3.058</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0042</v>
+        <v>0.8512999999999999</v>
       </c>
       <c r="V3" t="n">
-        <v>75.9474</v>
+        <v>0.8509</v>
       </c>
       <c r="W3" t="n">
-        <v>21.4203</v>
+        <v>0.0385</v>
       </c>
       <c r="X3" t="n">
-        <v>97.7983</v>
+        <v>0.0828</v>
       </c>
       <c r="Y3" t="n">
-        <v>73.6207</v>
+        <v>0.0418</v>
       </c>
       <c r="Z3" t="n">
-        <v>3.6179</v>
+        <v>0.0104</v>
       </c>
       <c r="AA3" t="n">
-        <v>1.1969</v>
+        <v>0.0034</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.9114</v>
+        <v>0.8497</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.063</v>
+        <v>0.0413</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.0885</v>
+        <v>0.0236</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.016</v>
+        <v>0.0046</v>
       </c>
       <c r="AF3" t="n">
-        <v>13.3971</v>
+        <v>3.7683</v>
       </c>
       <c r="AG3" t="n">
-        <v>6.3461</v>
+        <v>1.091</v>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
@@ -841,94 +841,94 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.8631</v>
+        <v>90.15000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.037</v>
+        <v>45.7847</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0274</v>
+        <v>109.4879</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0064</v>
+        <v>62.308</v>
       </c>
       <c r="H4" t="n">
-        <v>4.2772</v>
+        <v>4.893</v>
       </c>
       <c r="I4" t="n">
-        <v>1.0262</v>
+        <v>1.4594</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8611</v>
+        <v>0.9065</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0385</v>
+        <v>0.0311</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0367</v>
+        <v>0.1101</v>
       </c>
       <c r="M4" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0114</v>
       </c>
       <c r="N4" t="n">
-        <v>5.7092</v>
+        <v>28.145</v>
       </c>
       <c r="O4" t="n">
-        <v>1.3328</v>
+        <v>12.4578</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8631</v>
+        <v>0.8636</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0355</v>
+        <v>0.0396</v>
       </c>
       <c r="R4" t="n">
-        <v>0.1081</v>
+        <v>0.027</v>
       </c>
       <c r="S4" t="n">
-        <v>0.0489</v>
+        <v>0.0067</v>
       </c>
       <c r="T4" t="n">
-        <v>0.0209</v>
+        <v>4.1963</v>
       </c>
       <c r="U4" t="n">
-        <v>0.0069</v>
+        <v>0.9523</v>
       </c>
       <c r="V4" t="n">
-        <v>85.65000000000001</v>
+        <v>0.8636</v>
       </c>
       <c r="W4" t="n">
-        <v>43.2828</v>
+        <v>0.0386</v>
       </c>
       <c r="X4" t="n">
-        <v>116.4277</v>
+        <v>0.0921</v>
       </c>
       <c r="Y4" t="n">
-        <v>69.68380000000001</v>
+        <v>0.0384</v>
       </c>
       <c r="Z4" t="n">
-        <v>4.884</v>
+        <v>0.0246</v>
       </c>
       <c r="AA4" t="n">
-        <v>1.4537</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.9036999999999999</v>
+        <v>0.8614000000000001</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.0326</v>
+        <v>0.0404</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.1218</v>
+        <v>0.0345</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.0162</v>
+        <v>0.0078</v>
       </c>
       <c r="AF4" t="n">
-        <v>32.0503</v>
+        <v>5.4096</v>
       </c>
       <c r="AG4" t="n">
-        <v>14.6117</v>
+        <v>1.3466</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -953,178 +953,96 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.8625</v>
+        <v>67.2</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0366</v>
+        <v>19.0639</v>
       </c>
       <c r="F5" t="n">
-        <v>0.019</v>
+        <v>68.643</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0035</v>
+        <v>51.7651</v>
       </c>
       <c r="H5" t="n">
-        <v>3.0539</v>
+        <v>2.061</v>
       </c>
       <c r="I5" t="n">
-        <v>0.9064</v>
+        <v>0.6554</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8595</v>
+        <v>0.9087</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0381</v>
+        <v>0.0265</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0237</v>
+        <v>0.0696</v>
       </c>
       <c r="M5" t="n">
-        <v>0.0052</v>
+        <v>0.0109</v>
       </c>
       <c r="N5" t="n">
-        <v>3.746</v>
+        <v>11.2968</v>
       </c>
       <c r="O5" t="n">
-        <v>0.9807</v>
+        <v>4.7719</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8626</v>
+        <v>0.8581</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.0371</v>
+        <v>0.0398</v>
       </c>
       <c r="R5" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0185</v>
       </c>
       <c r="S5" t="n">
-        <v>0.0537</v>
+        <v>0.0037</v>
       </c>
       <c r="T5" t="n">
-        <v>0.0108</v>
+        <v>2.9433</v>
       </c>
       <c r="U5" t="n">
-        <v>0.0024</v>
+        <v>0.8186</v>
       </c>
       <c r="V5" t="n">
-        <v>73.59999999999999</v>
+        <v>0.8591</v>
       </c>
       <c r="W5" t="n">
-        <v>25.5722</v>
+        <v>0.0388</v>
       </c>
       <c r="X5" t="n">
-        <v>87.9074</v>
+        <v>0.076</v>
       </c>
       <c r="Y5" t="n">
-        <v>66.932</v>
+        <v>0.0476</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.062</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.6278</v>
+        <v>0.0022</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.9087</v>
+        <v>0.8541</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.0249</v>
+        <v>0.0429</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.0795</v>
+        <v>0.0227</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.0188</v>
+        <v>0.0049</v>
       </c>
       <c r="AF5" t="n">
-        <v>12.3645</v>
+        <v>3.5882</v>
       </c>
       <c r="AG5" t="n">
-        <v>5.4597</v>
+        <v>0.9651999999999999</v>
       </c>
       <c r="AH5" t="inlineStr">
-        <is>
-          <t>MULTI_LABEL_CLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MULTI_LABEL_CLS</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>efficientnet_b0</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.8217</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="n">
-        <v>0.0213</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>2.1344</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="n">
-        <v>0.8217</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="n">
-        <v>0.0272</v>
-      </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
-        <v>2.7152</v>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="n">
-        <v>0.8217</v>
-      </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="n">
-        <v>44</v>
-      </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="n">
-        <v>25.3164</v>
-      </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="n">
-        <v>4.24</v>
-      </c>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="n">
-        <v>0.8333</v>
-      </c>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="n">
-        <v>0.0751</v>
-      </c>
-      <c r="AE6" t="inlineStr"/>
-      <c r="AF6" t="n">
-        <v>9.2143</v>
-      </c>
-      <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
         <is>
           <t>MULTI_LABEL_CLS</t>
         </is>

</xml_diff>